<commit_message>
Adiciona aba Capitais na projeção x2 de pedidos Nordeste
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EQxeMa493LnVLgiFiREJjT
</commit_message>
<xml_diff>
--- a/Pedidos_por_Cidade_UF_Nordeste_Ago26_x2.xlsx
+++ b/Pedidos_por_Cidade_UF_Nordeste_Ago26_x2.xlsx
@@ -9,6 +9,7 @@
   </bookViews>
   <sheets>
     <sheet name="Pedidos por Cidade e UF" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Capitais" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Pedidos por Cidade e UF'!$I$5:$N$728</definedName>
@@ -23,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1662" uniqueCount="743">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1692" uniqueCount="751">
   <si>
     <t xml:space="preserve">Projeção de pedidos (×2) por estado e cidade – base Nordeste, agosto/2026</t>
   </si>
@@ -2252,6 +2253,30 @@
   </si>
   <si>
     <t xml:space="preserve">SAO MIGUEL DO ALEIXO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pedidos nas capitais do Nordeste – projeção (×2), base agosto/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valores vêm da aba 'Pedidos por Cidade e UF' e acompanham o fator de multiplicação da célula C3 de lá.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capital</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pedidos do estado (×2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% da capital no estado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pedidos no interior (×2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% do total Nordeste</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9 capitais</t>
   </si>
 </sst>
 </file>
@@ -21771,7 +21796,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{688BAC26-56FC-4E5B-A165-438C3967141F}</x14:id>
+          <x14:id>{F3FDE6DC-BD39-4050-A2CA-B27C4C10A590}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -21785,7 +21810,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{20FAF215-59E5-48C3-BB6C-DA6A00E64CD0}</x14:id>
+          <x14:id>{F7E07513-85F0-473F-BCD5-17B0B0FD0014}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -21802,7 +21827,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{688BAC26-56FC-4E5B-A165-438C3967141F}">
+          <x14:cfRule type="dataBar" id="{F3FDE6DC-BD39-4050-A2CA-B27C4C10A590}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -21815,7 +21840,7 @@
           <xm:sqref>D20:D109</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{20FAF215-59E5-48C3-BB6C-DA6A00E64CD0}">
+          <x14:cfRule type="dataBar" id="{F7E07513-85F0-473F-BCD5-17B0B0FD0014}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -21831,4 +21856,448 @@
     </ext>
   </extLst>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:H14"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="5" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>745</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>746</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>747</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>748</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>749</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C5" s="7" t="n">
+        <f aca="false">SUMIFS('Pedidos por Cidade e UF'!$K$6:$K$728,'Pedidos por Cidade e UF'!$I$6:$I$728,A5,'Pedidos por Cidade e UF'!$J$6:$J$728,B5)</f>
+        <v>596</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <f aca="false">SUMIFS('Pedidos por Cidade e UF'!$N$6:$N$728,'Pedidos por Cidade e UF'!$I$6:$I$728,A5,'Pedidos por Cidade e UF'!$J$6:$J$728,B5)</f>
+        <v>298</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <f aca="false">SUMIFS('Pedidos por Cidade e UF'!$K$6:$K$728,'Pedidos por Cidade e UF'!$I$6:$I$728,A5)</f>
+        <v>1746</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <f aca="false">IF(E5=0,0,C5/E5)</f>
+        <v>0.34135166093929</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <f aca="false">E5-C5</f>
+        <v>1150</v>
+      </c>
+      <c r="H5" s="8" t="n">
+        <f aca="false">C5/$E$14</f>
+        <v>0.102440701271915</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="C6" s="7" t="n">
+        <f aca="false">SUMIFS('Pedidos por Cidade e UF'!$K$6:$K$728,'Pedidos por Cidade e UF'!$I$6:$I$728,A6,'Pedidos por Cidade e UF'!$J$6:$J$728,B6)</f>
+        <v>286</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <f aca="false">SUMIFS('Pedidos por Cidade e UF'!$N$6:$N$728,'Pedidos por Cidade e UF'!$I$6:$I$728,A6,'Pedidos por Cidade e UF'!$J$6:$J$728,B6)</f>
+        <v>143</v>
+      </c>
+      <c r="E6" s="7" t="n">
+        <f aca="false">SUMIFS('Pedidos por Cidade e UF'!$K$6:$K$728,'Pedidos por Cidade e UF'!$I$6:$I$728,A6)</f>
+        <v>1074</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <f aca="false">IF(E6=0,0,C6/E6)</f>
+        <v>0.266294227188082</v>
+      </c>
+      <c r="G6" s="7" t="n">
+        <f aca="false">E6-C6</f>
+        <v>788</v>
+      </c>
+      <c r="H6" s="8" t="n">
+        <f aca="false">C6/$E$14</f>
+        <v>0.0491577861808182</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <f aca="false">SUMIFS('Pedidos por Cidade e UF'!$K$6:$K$728,'Pedidos por Cidade e UF'!$I$6:$I$728,A7,'Pedidos por Cidade e UF'!$J$6:$J$728,B7)</f>
+        <v>382</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <f aca="false">SUMIFS('Pedidos por Cidade e UF'!$N$6:$N$728,'Pedidos por Cidade e UF'!$I$6:$I$728,A7,'Pedidos por Cidade e UF'!$J$6:$J$728,B7)</f>
+        <v>191</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <f aca="false">SUMIFS('Pedidos por Cidade e UF'!$K$6:$K$728,'Pedidos por Cidade e UF'!$I$6:$I$728,A7)</f>
+        <v>732</v>
+      </c>
+      <c r="F7" s="8" t="n">
+        <f aca="false">IF(E7=0,0,C7/E7)</f>
+        <v>0.521857923497268</v>
+      </c>
+      <c r="G7" s="7" t="n">
+        <f aca="false">E7-C7</f>
+        <v>350</v>
+      </c>
+      <c r="H7" s="8" t="n">
+        <f aca="false">C7/$E$14</f>
+        <v>0.0656583018219319</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C8" s="7" t="n">
+        <f aca="false">SUMIFS('Pedidos por Cidade e UF'!$K$6:$K$728,'Pedidos por Cidade e UF'!$I$6:$I$728,A8,'Pedidos por Cidade e UF'!$J$6:$J$728,B8)</f>
+        <v>138</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <f aca="false">SUMIFS('Pedidos por Cidade e UF'!$N$6:$N$728,'Pedidos por Cidade e UF'!$I$6:$I$728,A8,'Pedidos por Cidade e UF'!$J$6:$J$728,B8)</f>
+        <v>69</v>
+      </c>
+      <c r="E8" s="7" t="n">
+        <f aca="false">SUMIFS('Pedidos por Cidade e UF'!$K$6:$K$728,'Pedidos por Cidade e UF'!$I$6:$I$728,A8)</f>
+        <v>638</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <f aca="false">IF(E8=0,0,C8/E8)</f>
+        <v>0.216300940438871</v>
+      </c>
+      <c r="G8" s="7" t="n">
+        <f aca="false">E8-C8</f>
+        <v>500</v>
+      </c>
+      <c r="H8" s="8" t="n">
+        <f aca="false">C8/$E$14</f>
+        <v>0.0237194912341011</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="7" t="n">
+        <f aca="false">SUMIFS('Pedidos por Cidade e UF'!$K$6:$K$728,'Pedidos por Cidade e UF'!$I$6:$I$728,A9,'Pedidos por Cidade e UF'!$J$6:$J$728,B9)</f>
+        <v>228</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <f aca="false">SUMIFS('Pedidos por Cidade e UF'!$N$6:$N$728,'Pedidos por Cidade e UF'!$I$6:$I$728,A9,'Pedidos por Cidade e UF'!$J$6:$J$728,B9)</f>
+        <v>114</v>
+      </c>
+      <c r="E9" s="7" t="n">
+        <f aca="false">SUMIFS('Pedidos por Cidade e UF'!$K$6:$K$728,'Pedidos por Cidade e UF'!$I$6:$I$728,A9)</f>
+        <v>462</v>
+      </c>
+      <c r="F9" s="8" t="n">
+        <f aca="false">IF(E9=0,0,C9/E9)</f>
+        <v>0.493506493506494</v>
+      </c>
+      <c r="G9" s="7" t="n">
+        <f aca="false">E9-C9</f>
+        <v>234</v>
+      </c>
+      <c r="H9" s="8" t="n">
+        <f aca="false">C9/$E$14</f>
+        <v>0.0391887246476452</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="C10" s="7" t="n">
+        <f aca="false">SUMIFS('Pedidos por Cidade e UF'!$K$6:$K$728,'Pedidos por Cidade e UF'!$I$6:$I$728,A10,'Pedidos por Cidade e UF'!$J$6:$J$728,B10)</f>
+        <v>124</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <f aca="false">SUMIFS('Pedidos por Cidade e UF'!$N$6:$N$728,'Pedidos por Cidade e UF'!$I$6:$I$728,A10,'Pedidos por Cidade e UF'!$J$6:$J$728,B10)</f>
+        <v>62</v>
+      </c>
+      <c r="E10" s="7" t="n">
+        <f aca="false">SUMIFS('Pedidos por Cidade e UF'!$K$6:$K$728,'Pedidos por Cidade e UF'!$I$6:$I$728,A10)</f>
+        <v>346</v>
+      </c>
+      <c r="F10" s="8" t="n">
+        <f aca="false">IF(E10=0,0,C10/E10)</f>
+        <v>0.358381502890173</v>
+      </c>
+      <c r="G10" s="7" t="n">
+        <f aca="false">E10-C10</f>
+        <v>222</v>
+      </c>
+      <c r="H10" s="8" t="n">
+        <f aca="false">C10/$E$14</f>
+        <v>0.0213131660364386</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="C11" s="7" t="n">
+        <f aca="false">SUMIFS('Pedidos por Cidade e UF'!$K$6:$K$728,'Pedidos por Cidade e UF'!$I$6:$I$728,A11,'Pedidos por Cidade e UF'!$J$6:$J$728,B11)</f>
+        <v>142</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <f aca="false">SUMIFS('Pedidos por Cidade e UF'!$N$6:$N$728,'Pedidos por Cidade e UF'!$I$6:$I$728,A11,'Pedidos por Cidade e UF'!$J$6:$J$728,B11)</f>
+        <v>71</v>
+      </c>
+      <c r="E11" s="7" t="n">
+        <f aca="false">SUMIFS('Pedidos por Cidade e UF'!$K$6:$K$728,'Pedidos por Cidade e UF'!$I$6:$I$728,A11)</f>
+        <v>326</v>
+      </c>
+      <c r="F11" s="8" t="n">
+        <f aca="false">IF(E11=0,0,C11/E11)</f>
+        <v>0.43558282208589</v>
+      </c>
+      <c r="G11" s="7" t="n">
+        <f aca="false">E11-C11</f>
+        <v>184</v>
+      </c>
+      <c r="H11" s="8" t="n">
+        <f aca="false">C11/$E$14</f>
+        <v>0.0244070127191475</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="C12" s="7" t="n">
+        <f aca="false">SUMIFS('Pedidos por Cidade e UF'!$K$6:$K$728,'Pedidos por Cidade e UF'!$I$6:$I$728,A12,'Pedidos por Cidade e UF'!$J$6:$J$728,B12)</f>
+        <v>114</v>
+      </c>
+      <c r="D12" s="7" t="n">
+        <f aca="false">SUMIFS('Pedidos por Cidade e UF'!$N$6:$N$728,'Pedidos por Cidade e UF'!$I$6:$I$728,A12,'Pedidos por Cidade e UF'!$J$6:$J$728,B12)</f>
+        <v>57</v>
+      </c>
+      <c r="E12" s="7" t="n">
+        <f aca="false">SUMIFS('Pedidos por Cidade e UF'!$K$6:$K$728,'Pedidos por Cidade e UF'!$I$6:$I$728,A12)</f>
+        <v>270</v>
+      </c>
+      <c r="F12" s="8" t="n">
+        <f aca="false">IF(E12=0,0,C12/E12)</f>
+        <v>0.422222222222222</v>
+      </c>
+      <c r="G12" s="7" t="n">
+        <f aca="false">E12-C12</f>
+        <v>156</v>
+      </c>
+      <c r="H12" s="8" t="n">
+        <f aca="false">C12/$E$14</f>
+        <v>0.0195943623238226</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="C13" s="7" t="n">
+        <f aca="false">SUMIFS('Pedidos por Cidade e UF'!$K$6:$K$728,'Pedidos por Cidade e UF'!$I$6:$I$728,A13,'Pedidos por Cidade e UF'!$J$6:$J$728,B13)</f>
+        <v>72</v>
+      </c>
+      <c r="D13" s="7" t="n">
+        <f aca="false">SUMIFS('Pedidos por Cidade e UF'!$N$6:$N$728,'Pedidos por Cidade e UF'!$I$6:$I$728,A13,'Pedidos por Cidade e UF'!$J$6:$J$728,B13)</f>
+        <v>36</v>
+      </c>
+      <c r="E13" s="7" t="n">
+        <f aca="false">SUMIFS('Pedidos por Cidade e UF'!$K$6:$K$728,'Pedidos por Cidade e UF'!$I$6:$I$728,A13)</f>
+        <v>224</v>
+      </c>
+      <c r="F13" s="8" t="n">
+        <f aca="false">IF(E13=0,0,C13/E13)</f>
+        <v>0.321428571428571</v>
+      </c>
+      <c r="G13" s="7" t="n">
+        <f aca="false">E13-C13</f>
+        <v>152</v>
+      </c>
+      <c r="H13" s="8" t="n">
+        <f aca="false">C13/$E$14</f>
+        <v>0.0123753867308353</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>750</v>
+      </c>
+      <c r="C14" s="14" t="n">
+        <f aca="false">SUM(C5:C13)</f>
+        <v>2082</v>
+      </c>
+      <c r="D14" s="14" t="n">
+        <f aca="false">SUM(D5:D13)</f>
+        <v>1041</v>
+      </c>
+      <c r="E14" s="14" t="n">
+        <f aca="false">SUM(E5:E13)</f>
+        <v>5818</v>
+      </c>
+      <c r="F14" s="15" t="n">
+        <f aca="false">IF(E14=0,0,C14/E14)</f>
+        <v>0.357854932966655</v>
+      </c>
+      <c r="G14" s="14" t="n">
+        <f aca="false">SUM(G5:G13)</f>
+        <v>3736</v>
+      </c>
+      <c r="H14" s="15" t="n">
+        <f aca="false">C14/$E$14</f>
+        <v>0.357854932966655</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="C5:C13">
+    <cfRule type="dataBar" priority="2">
+      <dataBar showValue="1" minLength="10" maxLength="90">
+        <cfvo type="num" val="0"/>
+        <cfvo type="max" val="0"/>
+        <color rgb="FF8EA9DB"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{A5B7B3AA-DEC7-439F-87A8-6E84F0A3447C}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F5:F13">
+    <cfRule type="dataBar" priority="3">
+      <dataBar showValue="1" minLength="10" maxLength="90">
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFA9D08E"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{901BD79D-BB77-4488-8A5A-609E2CA1C3F3}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{A5B7B3AA-DEC7-439F-87A8-6E84F0A3447C}">
+            <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
+              <x14:cfvo type="num">
+                <xm:f>0</xm:f>
+              </x14:cfvo>
+              <x14:cfvo type="max"/>
+              <x14:negativeFillColor rgb="FF8EA9DB"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>C5:C13</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{901BD79D-BB77-4488-8A5A-609E2CA1C3F3}">
+            <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
+              <x14:cfvo type="num">
+                <xm:f>0</xm:f>
+              </x14:cfvo>
+              <x14:cfvo type="num">
+                <xm:f>1</xm:f>
+              </x14:cfvo>
+              <x14:negativeFillColor rgb="FFA9D08E"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>F5:F13</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
+</worksheet>
 </file>
</xml_diff>